<commit_message>
Remove distribution type for end activity input.
</commit_message>
<xml_diff>
--- a/resources/Modelo - Atividade e Riscos (Monte Carlo).xlsx
+++ b/resources/Modelo - Atividade e Riscos (Monte Carlo).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b808ff425a94bbdc/Documents/Faculdade/Iniciação Científica/ARNA_UFPE/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{DA02E661-AE3D-4C1E-B96A-B0C0DA20CB68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{867AB3C8-3C59-4523-86B1-E5813294B518}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{DA02E661-AE3D-4C1E-B96A-B0C0DA20CB68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CDBC559A-747A-4CBD-8289-FF64092B487B}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="1100" windowWidth="14400" windowHeight="7270" xr2:uid="{7EB555F7-2C2B-4388-8B33-737FD34076B1}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7EB555F7-2C2B-4388-8B33-737FD34076B1}"/>
   </bookViews>
   <sheets>
     <sheet name="Atividades" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="38">
   <si>
     <t>Tipo</t>
   </si>
@@ -248,10 +248,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -963,9 +959,7 @@
       <c r="C10" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="6" t="s">
-        <v>19</v>
-      </c>
+      <c r="D10" s="6"/>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>

</xml_diff>

<commit_message>
Update MC xlsx model.
</commit_message>
<xml_diff>
--- a/resources/Modelo - Atividade e Riscos (Monte Carlo).xlsx
+++ b/resources/Modelo - Atividade e Riscos (Monte Carlo).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b808ff425a94bbdc/Documents/Faculdade/Iniciação Científica/ARNA_UFPE/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{DA02E661-AE3D-4C1E-B96A-B0C0DA20CB68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CDBC559A-747A-4CBD-8289-FF64092B487B}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="13_ncr:1_{DA02E661-AE3D-4C1E-B96A-B0C0DA20CB68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48410181-3A5E-4AE8-A8EC-B424626CEB83}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7EB555F7-2C2B-4388-8B33-737FD34076B1}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{7EB555F7-2C2B-4388-8B33-737FD34076B1}"/>
   </bookViews>
   <sheets>
     <sheet name="Atividades" sheetId="1" r:id="rId1"/>
@@ -34,10 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="38">
-  <si>
-    <t>Tipo</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="35">
   <si>
     <t>ID</t>
   </si>
@@ -48,33 +45,15 @@
     <t>Tipo de Distribuicao</t>
   </si>
   <si>
-    <t>Tempo Otimista</t>
-  </si>
-  <si>
-    <t>Tempo Provavel</t>
-  </si>
-  <si>
-    <t>Tempo Pessimista</t>
-  </si>
-  <si>
     <t>Tempo Minimo</t>
   </si>
   <si>
-    <t>Tempo Moda</t>
-  </si>
-  <si>
     <t>Tempo Maximo</t>
   </si>
   <si>
     <t>Tempo Medio</t>
   </si>
   <si>
-    <t>Custo</t>
-  </si>
-  <si>
-    <t>Probabilidade</t>
-  </si>
-  <si>
     <t>Atividades Afetadas</t>
   </si>
   <si>
@@ -87,18 +66,12 @@
     <t>Atraso Maximo</t>
   </si>
   <si>
-    <t>Descricao</t>
-  </si>
-  <si>
     <t>Atividade</t>
   </si>
   <si>
     <t>beta_pert</t>
   </si>
   <si>
-    <t>descricao da atividade</t>
-  </si>
-  <si>
     <t>triangular</t>
   </si>
   <si>
@@ -148,6 +121,24 @@
   </si>
   <si>
     <t>Custo Fixo Adicional</t>
+  </si>
+  <si>
+    <t>Tipo de Risco</t>
+  </si>
+  <si>
+    <t>Probabilidade do Risco Ocorrer</t>
+  </si>
+  <si>
+    <t>Custo Variavel Adicional</t>
+  </si>
+  <si>
+    <t>Desvio Padrao</t>
+  </si>
+  <si>
+    <t>Probabilidade do Tempo Otimista</t>
+  </si>
+  <si>
+    <t>Probabilidade do Atraso Otimista</t>
   </si>
 </sst>
 </file>
@@ -248,6 +239,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -577,8 +572,9 @@
     <col min="5" max="5" width="15.26953125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.7265625" customWidth="1"/>
     <col min="7" max="8" width="16" customWidth="1"/>
+    <col min="9" max="9" width="29.26953125" customWidth="1"/>
     <col min="10" max="10" width="10.54296875" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="12" max="12" width="14" customWidth="1"/>
     <col min="14" max="14" width="22.453125" customWidth="1"/>
     <col min="15" max="15" width="16.26953125" customWidth="1"/>
     <col min="16" max="16" width="12.81640625" bestFit="1" customWidth="1"/>
@@ -587,46 +583,37 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="B1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="D1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="E1" s="6" t="s">
         <v>3</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>4</v>
       </c>
       <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>8</v>
+        <v>33</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="M1" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="N1" s="6" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="O1" s="6"/>
       <c r="P1" s="3"/>
@@ -635,14 +622,14 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B2" s="6">
         <v>1</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E2" s="6">
         <v>3</v>
@@ -653,17 +640,10 @@
       <c r="G2" s="6">
         <v>8</v>
       </c>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6">
+      <c r="J2" s="6">
         <v>100</v>
       </c>
-      <c r="M2" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="N2" s="6">
+      <c r="K2" s="6">
         <v>1.3</v>
       </c>
       <c r="O2" s="6"/>
@@ -673,7 +653,7 @@
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B3" s="6">
         <v>2</v>
@@ -682,28 +662,21 @@
         <v>1</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6">
+        <v>12</v>
+      </c>
+      <c r="E3" s="6">
         <v>3</v>
       </c>
-      <c r="I3" s="6">
+      <c r="F3" s="6">
         <v>6</v>
       </c>
+      <c r="G3" s="6">
+        <v>10</v>
+      </c>
       <c r="J3" s="6">
-        <v>10</v>
-      </c>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6">
         <v>0</v>
       </c>
-      <c r="M3" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="N3" s="6">
+      <c r="K3" s="6">
         <v>0.2</v>
       </c>
       <c r="O3" s="6"/>
@@ -713,35 +686,28 @@
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B4" s="6">
         <v>3</v>
       </c>
       <c r="C4" s="6">
+        <v>2</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="6">
         <v>1</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" s="6"/>
       <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6">
-        <v>1</v>
-      </c>
-      <c r="I4" s="6"/>
+      <c r="G4" s="6">
+        <v>4</v>
+      </c>
       <c r="J4" s="6">
-        <v>4</v>
-      </c>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6">
         <v>0</v>
       </c>
-      <c r="M4" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="N4" s="6">
+      <c r="K4" s="6">
         <v>0.2</v>
       </c>
       <c r="O4" s="6"/>
@@ -751,7 +717,7 @@
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B5" s="6">
         <v>4</v>
@@ -760,28 +726,20 @@
         <v>2</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" s="6">
-        <v>4</v>
-      </c>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6">
-        <v>8</v>
-      </c>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
+        <v>14</v>
+      </c>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6">
+        <v>6</v>
+      </c>
+      <c r="G5" s="6"/>
+      <c r="H5">
+        <v>0.2</v>
+      </c>
+      <c r="J5" s="6">
+        <v>0</v>
+      </c>
       <c r="K5" s="6">
-        <v>6</v>
-      </c>
-      <c r="L5" s="6">
-        <v>0</v>
-      </c>
-      <c r="M5" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="N5" s="6">
         <v>0.2</v>
       </c>
       <c r="O5" s="6"/>
@@ -791,16 +749,14 @@
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B6" s="6">
         <v>5</v>
       </c>
-      <c r="C6" s="6">
-        <v>2</v>
-      </c>
+      <c r="C6" s="6"/>
       <c r="D6" s="6" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E6" s="6">
         <v>8</v>
@@ -811,17 +767,10 @@
       <c r="G6" s="6">
         <v>12</v>
       </c>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6">
+      <c r="J6" s="6">
         <v>0</v>
       </c>
-      <c r="M6" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="N6" s="6">
+      <c r="K6" s="6">
         <v>0.2</v>
       </c>
       <c r="O6" s="6"/>
@@ -831,7 +780,7 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B7" s="6">
         <v>6</v>
@@ -840,7 +789,7 @@
         <v>3</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E7" s="6">
         <v>3</v>
@@ -851,17 +800,10 @@
       <c r="G7" s="6">
         <v>6</v>
       </c>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6">
+      <c r="J7" s="6">
         <v>0</v>
       </c>
-      <c r="M7" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="N7" s="6">
+      <c r="K7" s="6">
         <v>0.2</v>
       </c>
       <c r="O7" s="6"/>
@@ -871,16 +813,16 @@
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B8" s="6">
         <v>7</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E8" s="6">
         <v>7</v>
@@ -891,17 +833,10 @@
       <c r="G8" s="6">
         <v>11</v>
       </c>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6">
+      <c r="J8" s="6">
         <v>0</v>
       </c>
-      <c r="M8" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="N8" s="6">
+      <c r="K8" s="6">
         <v>0.2</v>
       </c>
       <c r="O8" s="6"/>
@@ -911,7 +846,7 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B9" s="6">
         <v>8</v>
@@ -920,7 +855,7 @@
         <v>6</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E9" s="6">
         <v>3</v>
@@ -931,17 +866,10 @@
       <c r="G9" s="6">
         <v>6</v>
       </c>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="6"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="6">
+      <c r="J9" s="6">
         <v>0</v>
       </c>
-      <c r="M9" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="N9" s="6">
+      <c r="K9" s="6">
         <v>0.2</v>
       </c>
       <c r="O9" s="6"/>
@@ -951,30 +879,23 @@
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6">
+      <c r="J10" s="6">
         <v>0</v>
       </c>
-      <c r="M10" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="N10" s="6">
-        <v>0.2</v>
+      <c r="K10" s="6">
+        <v>0</v>
       </c>
       <c r="O10" s="6"/>
       <c r="P10" s="3"/>
@@ -989,11 +910,8 @@
       <c r="E11" s="6"/>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
       <c r="J11" s="6"/>
       <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
       <c r="M11" s="6"/>
       <c r="N11" s="6"/>
       <c r="O11" s="6"/>
@@ -1013,9 +931,7 @@
       <c r="F12" s="6"/>
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
       <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
       <c r="L12" s="6"/>
       <c r="M12" s="6"/>
       <c r="N12" s="6"/>
@@ -1035,9 +951,7 @@
       <c r="F13" s="6"/>
       <c r="G13" s="6"/>
       <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
       <c r="J13" s="6"/>
-      <c r="K13" s="6"/>
       <c r="L13" s="6"/>
       <c r="M13" s="6"/>
       <c r="N13" s="6"/>
@@ -1057,9 +971,7 @@
       <c r="F14" s="6"/>
       <c r="G14" s="6"/>
       <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
       <c r="J14" s="6"/>
-      <c r="K14" s="6"/>
       <c r="L14" s="6"/>
       <c r="M14" s="6"/>
       <c r="N14" s="6"/>
@@ -1079,9 +991,7 @@
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
       <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
@@ -1108,152 +1018,156 @@
     <col min="1" max="1" width="10.1796875" customWidth="1"/>
     <col min="2" max="2" width="10.26953125" customWidth="1"/>
     <col min="3" max="3" width="18.1796875" customWidth="1"/>
-    <col min="4" max="4" width="13.81640625" customWidth="1"/>
-    <col min="11" max="11" width="20.7265625" customWidth="1"/>
+    <col min="4" max="4" width="18.26953125" customWidth="1"/>
+    <col min="5" max="5" width="21" customWidth="1"/>
+    <col min="6" max="6" width="17.453125" customWidth="1"/>
+    <col min="7" max="7" width="26.08984375" customWidth="1"/>
+    <col min="8" max="8" width="17.81640625" customWidth="1"/>
+    <col min="9" max="9" width="13.36328125" customWidth="1"/>
+    <col min="10" max="10" width="14.1796875" customWidth="1"/>
+    <col min="11" max="11" width="13.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="M1" s="6"/>
       <c r="N1" s="6"/>
     </row>
     <row r="2" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E2" s="6"/>
       <c r="F2" s="6">
+        <v>2</v>
+      </c>
+      <c r="G2" s="6">
         <v>0.5</v>
       </c>
-      <c r="G2" s="6">
+      <c r="H2" s="6">
         <v>1</v>
       </c>
-      <c r="H2" s="6">
+      <c r="I2" s="6">
         <v>3</v>
       </c>
-      <c r="I2" s="6">
+      <c r="J2" s="6">
         <v>4</v>
       </c>
-      <c r="J2" s="6">
+      <c r="K2" s="6">
         <v>5</v>
-      </c>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6">
-        <v>2</v>
       </c>
       <c r="M2" s="6"/>
       <c r="N2" s="7"/>
     </row>
     <row r="3" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="6">
+        <v>2</v>
+      </c>
+      <c r="G3" s="6">
         <v>0.3</v>
       </c>
-      <c r="G3" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="H3" s="6">
+      <c r="H3" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" s="6">
         <v>0.3</v>
       </c>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6">
+      <c r="J3" s="6"/>
+      <c r="K3" s="6">
         <v>0.5</v>
-      </c>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6">
-        <v>2</v>
       </c>
       <c r="M3" s="6"/>
       <c r="N3" s="7"/>
     </row>
     <row r="4" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="L4" s="5"/>
+      <c r="F4" s="5"/>
       <c r="M4" s="5"/>
       <c r="N4" s="5"/>
     </row>
     <row r="5" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="L5" s="5"/>
+      <c r="F5" s="5"/>
       <c r="M5" s="5"/>
       <c r="N5" s="5"/>
     </row>
     <row r="6" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="L6" s="5"/>
+      <c r="F6" s="5"/>
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
     </row>
     <row r="7" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="L7" s="5"/>
+      <c r="F7" s="5"/>
       <c r="M7" s="5"/>
       <c r="N7" s="5"/>
     </row>
     <row r="8" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="L8" s="5"/>
+      <c r="F8" s="5"/>
       <c r="M8" s="5"/>
       <c r="N8" s="5"/>
     </row>
     <row r="9" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="L9" s="5"/>
+      <c r="F9" s="5"/>
       <c r="M9" s="5"/>
       <c r="N9" s="5"/>
     </row>
     <row r="10" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="L10" s="5"/>
+      <c r="F10" s="5"/>
       <c r="M10" s="5"/>
       <c r="N10" s="5"/>
     </row>
@@ -1267,28 +1181,28 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="C13" s="2"/>
-      <c r="L13" s="4"/>
+      <c r="F13" s="4"/>
       <c r="M13" s="4"/>
       <c r="N13" s="4"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="L14" s="4"/>
+      <c r="F14" s="4"/>
       <c r="M14" s="4"/>
       <c r="N14" s="4"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="C15" s="3"/>
-      <c r="L15" s="4"/>
+      <c r="F15" s="4"/>
       <c r="M15" s="4"/>
       <c r="N15" s="4"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="L16" s="4"/>
+      <c r="F16" s="4"/>
       <c r="M16" s="4"/>
       <c r="N16" s="4"/>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="L17" s="4"/>
+      <c r="F17" s="4"/>
       <c r="M17" s="4"/>
       <c r="N17" s="4"/>
     </row>
@@ -1316,7 +1230,6 @@
       <c r="I21" s="4"/>
       <c r="J21" s="4"/>
       <c r="K21" s="4"/>
-      <c r="L21" s="4"/>
       <c r="M21" s="4"/>
       <c r="N21" s="4"/>
       <c r="O21" s="4"/>
@@ -1335,7 +1248,6 @@
       <c r="I22" s="4"/>
       <c r="J22" s="4"/>
       <c r="K22" s="4"/>
-      <c r="L22" s="4"/>
       <c r="M22" s="4"/>
       <c r="N22" s="4"/>
       <c r="O22" s="4"/>
@@ -1343,7 +1255,7 @@
       <c r="Q22" s="4"/>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="L23" s="4"/>
+      <c r="F23" s="4"/>
       <c r="M23" s="4"/>
       <c r="N23" s="4"/>
     </row>

</xml_diff>

<commit_message>
New column name for .xlsx MC model.
</commit_message>
<xml_diff>
--- a/resources/Modelo - Atividade e Riscos (Monte Carlo).xlsx
+++ b/resources/Modelo - Atividade e Riscos (Monte Carlo).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b808ff425a94bbdc/Documents/Faculdade/Iniciação Científica/ARNA_UFPE/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="58" documentId="13_ncr:1_{DA02E661-AE3D-4C1E-B96A-B0C0DA20CB68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48410181-3A5E-4AE8-A8EC-B424626CEB83}"/>
+  <xr:revisionPtr revIDLastSave="77" documentId="13_ncr:1_{DA02E661-AE3D-4C1E-B96A-B0C0DA20CB68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3709F80B-87F9-49D4-A54C-B02412F5A84C}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{7EB555F7-2C2B-4388-8B33-737FD34076B1}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="37">
   <si>
     <t>ID</t>
   </si>
@@ -51,9 +51,6 @@
     <t>Tempo Maximo</t>
   </si>
   <si>
-    <t>Tempo Medio</t>
-  </si>
-  <si>
     <t>Atividades Afetadas</t>
   </si>
   <si>
@@ -139,6 +136,15 @@
   </si>
   <si>
     <t>Probabilidade do Atraso Otimista</t>
+  </si>
+  <si>
+    <t>Tempo Mais Provavel</t>
+  </si>
+  <si>
+    <t>Media</t>
+  </si>
+  <si>
+    <t>Tipo de Distribuicao da Consequencia</t>
   </si>
 </sst>
 </file>
@@ -570,11 +576,12 @@
     <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.26953125" customWidth="1"/>
     <col min="5" max="5" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.7265625" customWidth="1"/>
-    <col min="7" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="29.26953125" customWidth="1"/>
-    <col min="10" max="10" width="10.54296875" customWidth="1"/>
-    <col min="12" max="12" width="14" customWidth="1"/>
+    <col min="6" max="6" width="19.1796875" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="29.26953125" customWidth="1"/>
+    <col min="11" max="11" width="10.54296875" customWidth="1"/>
+    <col min="13" max="13" width="14" customWidth="1"/>
     <col min="14" max="14" width="22.453125" customWidth="1"/>
     <col min="15" max="15" width="16.26953125" customWidth="1"/>
     <col min="16" max="16" width="12.81640625" bestFit="1" customWidth="1"/>
@@ -583,7 +590,7 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>0</v>
@@ -598,22 +605,25 @@
         <v>3</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>4</v>
       </c>
       <c r="H1" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="J1" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="I1" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="J1" s="6" t="s">
+      <c r="K1" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L1" s="6" t="s">
         <v>26</v>
-      </c>
-      <c r="K1" s="6" t="s">
-        <v>27</v>
       </c>
       <c r="O1" s="6"/>
       <c r="P1" s="3"/>
@@ -622,14 +632,14 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2" s="6">
         <v>1</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E2" s="6">
         <v>3</v>
@@ -640,10 +650,10 @@
       <c r="G2" s="6">
         <v>8</v>
       </c>
-      <c r="J2" s="6">
+      <c r="K2" s="6">
         <v>100</v>
       </c>
-      <c r="K2" s="6">
+      <c r="L2" s="6">
         <v>1.3</v>
       </c>
       <c r="O2" s="6"/>
@@ -653,7 +663,7 @@
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B3" s="6">
         <v>2</v>
@@ -662,7 +672,7 @@
         <v>1</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E3" s="6">
         <v>3</v>
@@ -673,10 +683,10 @@
       <c r="G3" s="6">
         <v>10</v>
       </c>
-      <c r="J3" s="6">
+      <c r="K3" s="6">
         <v>0</v>
       </c>
-      <c r="K3" s="6">
+      <c r="L3" s="6">
         <v>0.2</v>
       </c>
       <c r="O3" s="6"/>
@@ -686,7 +696,7 @@
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" s="6">
         <v>3</v>
@@ -695,7 +705,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E4" s="6">
         <v>1</v>
@@ -704,10 +714,10 @@
       <c r="G4" s="6">
         <v>4</v>
       </c>
-      <c r="J4" s="6">
+      <c r="K4" s="6">
         <v>0</v>
       </c>
-      <c r="K4" s="6">
+      <c r="L4" s="6">
         <v>0.2</v>
       </c>
       <c r="O4" s="6"/>
@@ -717,7 +727,7 @@
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B5" s="6">
         <v>4</v>
@@ -726,20 +736,21 @@
         <v>2</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E5" s="6"/>
-      <c r="F5" s="6">
-        <v>6</v>
-      </c>
+      <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5">
+        <v>6</v>
+      </c>
+      <c r="I5">
         <v>0.2</v>
       </c>
-      <c r="J5" s="6">
+      <c r="K5" s="6">
         <v>0</v>
       </c>
-      <c r="K5" s="6">
+      <c r="L5" s="6">
         <v>0.2</v>
       </c>
       <c r="O5" s="6"/>
@@ -749,14 +760,14 @@
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B6" s="6">
         <v>5</v>
       </c>
       <c r="C6" s="6"/>
       <c r="D6" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E6" s="6">
         <v>8</v>
@@ -767,10 +778,10 @@
       <c r="G6" s="6">
         <v>12</v>
       </c>
-      <c r="J6" s="6">
+      <c r="K6" s="6">
         <v>0</v>
       </c>
-      <c r="K6" s="6">
+      <c r="L6" s="6">
         <v>0.2</v>
       </c>
       <c r="O6" s="6"/>
@@ -780,7 +791,7 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7" s="6">
         <v>6</v>
@@ -789,7 +800,7 @@
         <v>3</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E7" s="6">
         <v>3</v>
@@ -800,10 +811,10 @@
       <c r="G7" s="6">
         <v>6</v>
       </c>
-      <c r="J7" s="6">
+      <c r="K7" s="6">
         <v>0</v>
       </c>
-      <c r="K7" s="6">
+      <c r="L7" s="6">
         <v>0.2</v>
       </c>
       <c r="O7" s="6"/>
@@ -813,16 +824,16 @@
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B8" s="6">
         <v>7</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E8" s="6">
         <v>7</v>
@@ -833,10 +844,10 @@
       <c r="G8" s="6">
         <v>11</v>
       </c>
-      <c r="J8" s="6">
+      <c r="K8" s="6">
         <v>0</v>
       </c>
-      <c r="K8" s="6">
+      <c r="L8" s="6">
         <v>0.2</v>
       </c>
       <c r="O8" s="6"/>
@@ -846,7 +857,7 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9" s="6">
         <v>8</v>
@@ -855,7 +866,7 @@
         <v>6</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E9" s="6">
         <v>3</v>
@@ -866,10 +877,10 @@
       <c r="G9" s="6">
         <v>6</v>
       </c>
-      <c r="J9" s="6">
+      <c r="K9" s="6">
         <v>0</v>
       </c>
-      <c r="K9" s="6">
+      <c r="L9" s="6">
         <v>0.2</v>
       </c>
       <c r="O9" s="6"/>
@@ -879,22 +890,22 @@
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="6" t="s">
         <v>16</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>17</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
-      <c r="J10" s="6">
+      <c r="K10" s="6">
         <v>0</v>
       </c>
-      <c r="K10" s="6">
+      <c r="L10" s="6">
         <v>0</v>
       </c>
       <c r="O10" s="6"/>
@@ -910,9 +921,8 @@
       <c r="E11" s="6"/>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
-      <c r="J11" s="6"/>
       <c r="K11" s="6"/>
-      <c r="M11" s="6"/>
+      <c r="L11" s="6"/>
       <c r="N11" s="6"/>
       <c r="O11" s="6"/>
       <c r="P11" s="3"/>
@@ -930,9 +940,8 @@
       <c r="E12" s="6"/>
       <c r="F12" s="6"/>
       <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="L12" s="6"/>
+      <c r="I12" s="6"/>
+      <c r="K12" s="6"/>
       <c r="M12" s="6"/>
       <c r="N12" s="6"/>
       <c r="O12" s="6"/>
@@ -950,9 +959,8 @@
       <c r="E13" s="6"/>
       <c r="F13" s="6"/>
       <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="J13" s="6"/>
-      <c r="L13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="K13" s="6"/>
       <c r="M13" s="6"/>
       <c r="N13" s="6"/>
       <c r="O13" s="6"/>
@@ -970,9 +978,8 @@
       <c r="E14" s="6"/>
       <c r="F14" s="6"/>
       <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="J14" s="6"/>
-      <c r="L14" s="6"/>
+      <c r="I14" s="6"/>
+      <c r="K14" s="6"/>
       <c r="M14" s="6"/>
       <c r="N14" s="6"/>
       <c r="O14" s="6"/>
@@ -990,9 +997,8 @@
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="L15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="K15" s="3"/>
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
       <c r="O15" s="3"/>
@@ -1018,10 +1024,10 @@
     <col min="1" max="1" width="10.1796875" customWidth="1"/>
     <col min="2" max="2" width="10.26953125" customWidth="1"/>
     <col min="3" max="3" width="18.1796875" customWidth="1"/>
-    <col min="4" max="4" width="18.26953125" customWidth="1"/>
+    <col min="4" max="4" width="26.54296875" customWidth="1"/>
     <col min="5" max="5" width="21" customWidth="1"/>
     <col min="6" max="6" width="17.453125" customWidth="1"/>
-    <col min="7" max="7" width="26.08984375" customWidth="1"/>
+    <col min="7" max="7" width="31.90625" customWidth="1"/>
     <col min="8" max="8" width="17.81640625" customWidth="1"/>
     <col min="9" max="9" width="13.36328125" customWidth="1"/>
     <col min="10" max="10" width="14.1796875" customWidth="1"/>
@@ -1030,63 +1036,63 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D1" s="6" t="s">
-        <v>2</v>
-      </c>
       <c r="E1" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="H1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="K1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="6" t="s">
-        <v>9</v>
-      </c>
       <c r="L1" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M1" s="6"/>
       <c r="N1" s="6"/>
     </row>
     <row r="2" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>19</v>
-      </c>
       <c r="C2" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>12</v>
+        <v>22</v>
+      </c>
+      <c r="D2" s="6">
+        <v>0.5</v>
       </c>
       <c r="E2" s="6"/>
       <c r="F2" s="6">
         <v>2</v>
       </c>
-      <c r="G2" s="6">
-        <v>0.5</v>
+      <c r="G2" s="6" t="s">
+        <v>11</v>
       </c>
       <c r="H2" s="6">
         <v>1</v>
@@ -1105,26 +1111,26 @@
     </row>
     <row r="3" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>13</v>
+        <v>21</v>
+      </c>
+      <c r="D3" s="6">
+        <v>0.3</v>
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="6">
         <v>2</v>
       </c>
-      <c r="G3" s="6">
-        <v>0.3</v>
+      <c r="G3" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I3" s="6">
         <v>0.3</v>

</xml_diff>

<commit_message>
Start point to MC.
</commit_message>
<xml_diff>
--- a/resources/Modelo - Atividade e Riscos (Monte Carlo).xlsx
+++ b/resources/Modelo - Atividade e Riscos (Monte Carlo).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b808ff425a94bbdc/Documents/Faculdade/Iniciação Científica/ARNA_UFPE/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="86" documentId="13_ncr:1_{DA02E661-AE3D-4C1E-B96A-B0C0DA20CB68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{79FBEE44-0125-4E89-95DD-5734F2E43875}"/>
+  <xr:revisionPtr revIDLastSave="91" documentId="13_ncr:1_{DA02E661-AE3D-4C1E-B96A-B0C0DA20CB68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{770EDF44-B255-479F-AC3D-5F1F12AEC8E3}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7EB555F7-2C2B-4388-8B33-737FD34076B1}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="38">
   <si>
     <t>ID</t>
   </si>
@@ -145,6 +145,9 @@
   </si>
   <si>
     <t>Probabilidade do Atraso Minimo</t>
+  </si>
+  <si>
+    <t>inicio</t>
   </si>
 </sst>
 </file>
@@ -631,30 +634,11 @@
       <c r="U1" s="4"/>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A2" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="6">
-        <v>1</v>
-      </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="6">
-        <v>3</v>
-      </c>
-      <c r="F2" s="6">
-        <v>5</v>
-      </c>
-      <c r="G2" s="6">
-        <v>8</v>
-      </c>
-      <c r="K2" s="6">
-        <v>100</v>
-      </c>
-      <c r="L2" s="6">
-        <v>1.3</v>
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>37</v>
       </c>
       <c r="O2" s="6"/>
       <c r="P2" s="3"/>
@@ -666,28 +650,28 @@
         <v>8</v>
       </c>
       <c r="B3" s="6">
-        <v>2</v>
-      </c>
-      <c r="C3" s="6">
         <v>1</v>
       </c>
+      <c r="C3" s="6" t="s">
+        <v>37</v>
+      </c>
       <c r="D3" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E3" s="6">
         <v>3</v>
       </c>
       <c r="F3" s="6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G3" s="6">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K3" s="6">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="L3" s="6">
-        <v>0.2</v>
+        <v>1.3</v>
       </c>
       <c r="O3" s="6"/>
       <c r="P3" s="3"/>
@@ -699,20 +683,22 @@
         <v>8</v>
       </c>
       <c r="B4" s="6">
+        <v>2</v>
+      </c>
+      <c r="C4" s="6">
+        <v>1</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="6">
         <v>3</v>
       </c>
-      <c r="C4" s="6">
-        <v>2</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="6">
-        <v>1</v>
-      </c>
-      <c r="F4" s="6"/>
+      <c r="F4" s="6">
+        <v>6</v>
+      </c>
       <c r="G4" s="6">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="K4" s="6">
         <v>0</v>
@@ -730,22 +716,20 @@
         <v>8</v>
       </c>
       <c r="B5" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C5" s="6">
         <v>2</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="6"/>
+        <v>11</v>
+      </c>
+      <c r="E5" s="6">
+        <v>1</v>
+      </c>
       <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5">
-        <v>6</v>
-      </c>
-      <c r="I5">
-        <v>0.2</v>
+      <c r="G5" s="6">
+        <v>4</v>
       </c>
       <c r="K5" s="6">
         <v>0</v>
@@ -763,20 +747,22 @@
         <v>8</v>
       </c>
       <c r="B6" s="6">
-        <v>5</v>
-      </c>
-      <c r="C6" s="6"/>
+        <v>4</v>
+      </c>
+      <c r="C6" s="6">
+        <v>2</v>
+      </c>
       <c r="D6" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" s="6">
-        <v>8</v>
-      </c>
-      <c r="F6" s="6">
-        <v>10</v>
-      </c>
-      <c r="G6" s="6">
         <v>12</v>
+      </c>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6">
+        <v>6</v>
+      </c>
+      <c r="I6">
+        <v>0.2</v>
       </c>
       <c r="K6" s="6">
         <v>0</v>
@@ -794,22 +780,22 @@
         <v>8</v>
       </c>
       <c r="B7" s="6">
-        <v>6</v>
-      </c>
-      <c r="C7" s="6">
-        <v>3</v>
+        <v>5</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>37</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E7" s="6">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F7" s="6">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G7" s="6">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="K7" s="6">
         <v>0</v>
@@ -827,22 +813,22 @@
         <v>8</v>
       </c>
       <c r="B8" s="6">
-        <v>7</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>13</v>
+        <v>6</v>
+      </c>
+      <c r="C8" s="6">
+        <v>3</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E8" s="6">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F8" s="6">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G8" s="6">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="K8" s="6">
         <v>0</v>
@@ -860,22 +846,22 @@
         <v>8</v>
       </c>
       <c r="B9" s="6">
-        <v>8</v>
-      </c>
-      <c r="C9" s="6">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>13</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E9" s="6">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F9" s="6">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G9" s="6">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="K9" s="6">
         <v>0</v>
@@ -892,21 +878,29 @@
       <c r="A10" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
+      <c r="B10" s="6">
+        <v>8</v>
+      </c>
+      <c r="C10" s="6">
+        <v>6</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" s="6">
+        <v>3</v>
+      </c>
+      <c r="F10" s="6">
+        <v>5</v>
+      </c>
+      <c r="G10" s="6">
+        <v>6</v>
+      </c>
       <c r="K10" s="6">
         <v>0</v>
       </c>
       <c r="L10" s="6">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="O10" s="6"/>
       <c r="P10" s="3"/>
@@ -914,15 +908,25 @@
       <c r="U10" s="4"/>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
+      <c r="A11" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>15</v>
+      </c>
       <c r="D11" s="6"/>
       <c r="E11" s="6"/>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
+      <c r="K11" s="6">
+        <v>0</v>
+      </c>
+      <c r="L11" s="6">
+        <v>0</v>
+      </c>
       <c r="N11" s="6"/>
       <c r="O11" s="6"/>
       <c r="P11" s="3"/>

</xml_diff>